<commit_message>
cdc_hypervisor_u2a16-CDC_Hypervisor_U2A16_Ver1.00r9 BSW https://gitlab.geniie.net/BSWPKG27/domain-controller/develop/projectdb/cdc_hypervisor_u2a16/-/releases/CDC_Hypervisor_U2A16_Ver1.00r9 2025/07/31リリース BEVCDCFD-1623
</commit_message>
<xml_diff>
--- a/src/PE0VM0/BSW/Communication/oXCAN/lib/oxcan_wrh_design.xlsx
+++ b/src/PE0VM0/BSW/Communication/oXCAN/lib/oxcan_wrh_design.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10001140895\Documents\Git\rh850_u2a\CANLpR_w_SecOC_v2\src\PE0VM0\BSW\Communication\oXCAN\lib\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10001140895\Documents\Git\rh850_u2a\SecOC-CANLpR-CANPNC_v1\src\PE0VM0\BSW\Communication\oXCAN\lib\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39EFB9A3-97C1-401D-B2DA-46D21887072D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F247A0-ACA0-42CB-9BB0-223FFC7EEE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -199,7 +199,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="113">
   <si>
     <t>EVENT</t>
     <phoneticPr fontId="3"/>
@@ -2256,19 +2256,15 @@
     <phoneticPr fontId="70"/>
   </si>
   <si>
-    <t>OXCAN_WRQH_EAS_TIM_OUT</t>
+    <t>OXCAN_WRQH_EAS_REQ_SS</t>
     <phoneticPr fontId="70"/>
   </si>
   <si>
-    <t>OXCAN_WRQH_EAS_REQ_STA</t>
+    <t>OXCAN_WRQH_EAS_REQ_ET</t>
     <phoneticPr fontId="70"/>
   </si>
   <si>
-    <t>\</t>
-    <phoneticPr fontId="70"/>
-  </si>
-  <si>
-    <t>OXCAN_WRQH_EAS_REQ_WKU</t>
+    <t>OXCAN_WRQH_EAS_TIMEOUT</t>
     <phoneticPr fontId="70"/>
   </si>
 </sst>
@@ -24179,18 +24175,18 @@
     <col min="9" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:15" ht="161.25">
+    <row r="3" spans="1:15" ht="159.75">
       <c r="A3" s="121" t="s">
         <v>109</v>
       </c>
       <c r="B3" s="121" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C3" s="121" t="s">
         <v>111</v>
       </c>
       <c r="D3" s="121" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E3" s="121"/>
       <c r="F3" s="123" t="s">
@@ -24222,11 +24218,11 @@
       <c r="B4" s="2">
         <v>0</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>112</v>
+      <c r="C4" s="2">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
       </c>
       <c r="F4" s="122" t="s">
         <v>108</v>

</xml_diff>